<commit_message>
Remove new app tag for non-applicable order types
</commit_message>
<xml_diff>
--- a/tests/fixtures/orderforms/1508.36.mip_rna.xlsx
+++ b/tests/fixtures/orderforms/1508.36.mip_rna.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/isakohlsson/dev/cg/tests/fixtures/orderforms/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9D268873-9034-FC49-902A-3AF43D4A39BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E575F973-FC4E-7846-B2DE-80FE2BEA8190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28800" yWindow="500" windowWidth="51200" windowHeight="28300" tabRatio="993" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15705,7 +15705,7 @@
         <v>722</v>
       </c>
       <c r="F17" s="67" t="s">
-        <v>712</v>
+        <v>460</v>
       </c>
       <c r="G17" s="68" t="s">
         <v>80</v>
@@ -16760,7 +16760,7 @@
         <v>729</v>
       </c>
       <c r="F18" s="67" t="s">
-        <v>460</v>
+        <v>551</v>
       </c>
       <c r="G18" s="68" t="s">
         <v>80</v>
@@ -17815,7 +17815,7 @@
         <v>732</v>
       </c>
       <c r="F19" s="67" t="s">
-        <v>551</v>
+        <v>460</v>
       </c>
       <c r="G19" s="68" t="s">
         <v>80</v>
@@ -18870,7 +18870,7 @@
         <v>735</v>
       </c>
       <c r="F20" s="67" t="s">
-        <v>712</v>
+        <v>551</v>
       </c>
       <c r="G20" s="68" t="s">
         <v>80</v>
@@ -22035,7 +22035,7 @@
         <v>744</v>
       </c>
       <c r="F23" s="67" t="s">
-        <v>712</v>
+        <v>460</v>
       </c>
       <c r="G23" s="68" t="s">
         <v>80</v>
@@ -23090,7 +23090,7 @@
         <v>747</v>
       </c>
       <c r="F24" s="67" t="s">
-        <v>460</v>
+        <v>551</v>
       </c>
       <c r="G24" s="68" t="s">
         <v>80</v>
@@ -24145,7 +24145,7 @@
         <v>750</v>
       </c>
       <c r="F25" s="67" t="s">
-        <v>551</v>
+        <v>460</v>
       </c>
       <c r="G25" s="68" t="s">
         <v>80</v>
@@ -25200,7 +25200,7 @@
         <v>753</v>
       </c>
       <c r="F26" s="67" t="s">
-        <v>712</v>
+        <v>551</v>
       </c>
       <c r="G26" s="68" t="s">
         <v>80</v>
@@ -27382,7 +27382,7 @@
         <v>762</v>
       </c>
       <c r="F29" s="67" t="s">
-        <v>712</v>
+        <v>460</v>
       </c>
       <c r="G29" s="68" t="s">
         <v>80</v>
@@ -28437,7 +28437,7 @@
         <v>765</v>
       </c>
       <c r="F30" s="67" t="s">
-        <v>460</v>
+        <v>551</v>
       </c>
       <c r="G30" s="68" t="s">
         <v>80</v>
@@ -29492,7 +29492,7 @@
         <v>768</v>
       </c>
       <c r="F31" s="67" t="s">
-        <v>551</v>
+        <v>460</v>
       </c>
       <c r="G31" s="68" t="s">
         <v>80</v>
@@ -30547,7 +30547,7 @@
         <v>771</v>
       </c>
       <c r="F32" s="67" t="s">
-        <v>712</v>
+        <v>551</v>
       </c>
       <c r="G32" s="68" t="s">
         <v>80</v>
@@ -33712,7 +33712,7 @@
         <v>780</v>
       </c>
       <c r="F35" s="67" t="s">
-        <v>712</v>
+        <v>460</v>
       </c>
       <c r="G35" s="68" t="s">
         <v>80</v>
@@ -34767,7 +34767,7 @@
         <v>783</v>
       </c>
       <c r="F36" s="67" t="s">
-        <v>460</v>
+        <v>551</v>
       </c>
       <c r="G36" s="68" t="s">
         <v>80</v>
@@ -34833,7 +34833,7 @@
         <v>786</v>
       </c>
       <c r="F37" s="67" t="s">
-        <v>551</v>
+        <v>460</v>
       </c>
       <c r="G37" s="68" t="s">
         <v>80</v>
@@ -34899,7 +34899,7 @@
         <v>789</v>
       </c>
       <c r="F38" s="67" t="s">
-        <v>712</v>
+        <v>551</v>
       </c>
       <c r="G38" s="68" t="s">
         <v>80</v>
@@ -37075,7 +37075,7 @@
         <v>798</v>
       </c>
       <c r="F41" s="67" t="s">
-        <v>712</v>
+        <v>460</v>
       </c>
       <c r="G41" s="68" t="s">
         <v>80</v>
@@ -38130,7 +38130,7 @@
         <v>801</v>
       </c>
       <c r="F42" s="67" t="s">
-        <v>460</v>
+        <v>551</v>
       </c>
       <c r="G42" s="68" t="s">
         <v>80</v>
@@ -39185,7 +39185,7 @@
         <v>804</v>
       </c>
       <c r="F43" s="67" t="s">
-        <v>551</v>
+        <v>460</v>
       </c>
       <c r="G43" s="68" t="s">
         <v>80</v>
@@ -40240,7 +40240,7 @@
         <v>807</v>
       </c>
       <c r="F44" s="67" t="s">
-        <v>712</v>
+        <v>551</v>
       </c>
       <c r="G44" s="68" t="s">
         <v>80</v>
@@ -43405,7 +43405,7 @@
         <v>816</v>
       </c>
       <c r="F47" s="67" t="s">
-        <v>712</v>
+        <v>460</v>
       </c>
       <c r="G47" s="68" t="s">
         <v>80</v>
@@ -44460,7 +44460,7 @@
         <v>819</v>
       </c>
       <c r="F48" s="67" t="s">
-        <v>460</v>
+        <v>551</v>
       </c>
       <c r="G48" s="68" t="s">
         <v>80</v>
@@ -45515,7 +45515,7 @@
         <v>822</v>
       </c>
       <c r="F49" s="67" t="s">
-        <v>551</v>
+        <v>460</v>
       </c>
       <c r="G49" s="68" t="s">
         <v>80</v>
@@ -46570,7 +46570,7 @@
         <v>825</v>
       </c>
       <c r="F50" s="67" t="s">
-        <v>712</v>
+        <v>551</v>
       </c>
       <c r="G50" s="68" t="s">
         <v>80</v>
@@ -48746,7 +48746,7 @@
         <v>834</v>
       </c>
       <c r="F53" s="67" t="s">
-        <v>712</v>
+        <v>460</v>
       </c>
       <c r="G53" s="68" t="s">
         <v>80</v>
@@ -49801,7 +49801,7 @@
         <v>837</v>
       </c>
       <c r="F54" s="67" t="s">
-        <v>460</v>
+        <v>551</v>
       </c>
       <c r="G54" s="68" t="s">
         <v>80</v>
@@ -50856,7 +50856,7 @@
         <v>840</v>
       </c>
       <c r="F55" s="67" t="s">
-        <v>551</v>
+        <v>460</v>
       </c>
       <c r="G55" s="68" t="s">
         <v>80</v>
@@ -51911,7 +51911,7 @@
         <v>843</v>
       </c>
       <c r="F56" s="67" t="s">
-        <v>712</v>
+        <v>551</v>
       </c>
       <c r="G56" s="68" t="s">
         <v>80</v>

</xml_diff>